<commit_message>
fix: code review changes
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/07-producer-certificate-submit.xlsx
+++ b/translations/welsh-translations/xlsx/07-producer-certificate-submit.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="110">
   <si>
     <t>Translator notes</t>
   </si>
@@ -103,27 +103,12 @@
     <t>If any information on this page is incorrect, contact the {{regulatorName}}:</t>
   </si>
   <si>
-    <t>compliance.components.overallStatus.recyclingObligationsHeading</t>
+    <t>compliance.components.obligationsTable.recyclingObligationsHeading</t>
   </si>
   <si>
     <t>Recycling obligations</t>
   </si>
   <si>
-    <t>compliance.components.overallStatus.overallMet</t>
-  </si>
-  <si>
-    <t>Recycling obligations have been met</t>
-  </si>
-  <si>
-    <t>compliance.components.overallStatus.overallNotMet</t>
-  </si>
-  <si>
-    <t>Recycling obligations have not been met</t>
-  </si>
-  <si>
-    <t>compliance.components.obligationsTable.recyclingObligationsHeading</t>
-  </si>
-  <si>
     <t>compliance.components.obligationsTable.tonnesNote</t>
   </si>
   <si>
@@ -172,6 +157,12 @@
     <t>Status</t>
   </si>
   <si>
+    <t>compliance.components.obligationsTable.notAvailableYet</t>
+  </si>
+  <si>
+    <t>Not available yet</t>
+  </si>
+  <si>
     <t>compliance.components.obligationsTable.material.paperComposite</t>
   </si>
   <si>
@@ -241,19 +232,19 @@
     <t>compliance.components.obligationsTable.obligationStatus.met</t>
   </si>
   <si>
-    <t>MET</t>
+    <t>Met</t>
   </si>
   <si>
     <t>compliance.components.obligationsTable.obligationStatus.notMet</t>
   </si>
   <si>
-    <t>NOT MET</t>
+    <t>Not met</t>
   </si>
   <si>
     <t>compliance.components.obligationsTable.obligationStatus.noDataYet</t>
   </si>
   <si>
-    <t>NO DATA YET</t>
+    <t>No data yet</t>
   </si>
   <si>
     <t>compliance.components.declaration.heading</t>
@@ -748,7 +739,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" hidden="1" customWidth="1"/>
@@ -1050,7 +1041,7 @@
         <v>11</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>13</v>
@@ -1061,7 +1052,7 @@
     </row>
     <row r="19" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>10</v>
@@ -1070,7 +1061,7 @@
         <v>11</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>13</v>
@@ -1081,7 +1072,7 @@
     </row>
     <row r="20" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>10</v>
@@ -1090,7 +1081,7 @@
         <v>11</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>13</v>
@@ -1101,7 +1092,7 @@
     </row>
     <row r="21" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>10</v>
@@ -1110,7 +1101,7 @@
         <v>11</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>13</v>
@@ -1121,7 +1112,7 @@
     </row>
     <row r="22" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>10</v>
@@ -1130,7 +1121,7 @@
         <v>11</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>13</v>
@@ -1141,7 +1132,7 @@
     </row>
     <row r="23" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>10</v>
@@ -1150,7 +1141,7 @@
         <v>11</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>13</v>
@@ -1161,7 +1152,7 @@
     </row>
     <row r="24" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>10</v>
@@ -1170,7 +1161,7 @@
         <v>11</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>13</v>
@@ -1181,7 +1172,7 @@
     </row>
     <row r="25" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>10</v>
@@ -1190,7 +1181,7 @@
         <v>11</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>13</v>
@@ -1201,7 +1192,7 @@
     </row>
     <row r="26" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>10</v>
@@ -1210,7 +1201,7 @@
         <v>11</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>13</v>
@@ -1221,7 +1212,7 @@
     </row>
     <row r="27" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>10</v>
@@ -1230,7 +1221,7 @@
         <v>11</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>13</v>
@@ -1241,7 +1232,7 @@
     </row>
     <row r="28" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>10</v>
@@ -1250,7 +1241,7 @@
         <v>11</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>13</v>
@@ -1261,7 +1252,7 @@
     </row>
     <row r="29" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>10</v>
@@ -1270,7 +1261,7 @@
         <v>11</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>13</v>
@@ -1281,7 +1272,7 @@
     </row>
     <row r="30" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>10</v>
@@ -1290,7 +1281,7 @@
         <v>11</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>13</v>
@@ -1301,7 +1292,7 @@
     </row>
     <row r="31" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>10</v>
@@ -1310,7 +1301,7 @@
         <v>11</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>13</v>
@@ -1321,7 +1312,7 @@
     </row>
     <row r="32" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>10</v>
@@ -1330,7 +1321,7 @@
         <v>11</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>13</v>
@@ -1341,7 +1332,7 @@
     </row>
     <row r="33" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>10</v>
@@ -1350,7 +1341,7 @@
         <v>11</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>13</v>
@@ -1361,7 +1352,7 @@
     </row>
     <row r="34" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>10</v>
@@ -1370,7 +1361,7 @@
         <v>11</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>13</v>
@@ -1381,7 +1372,7 @@
     </row>
     <row r="35" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>10</v>
@@ -1390,7 +1381,7 @@
         <v>11</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>13</v>
@@ -1401,7 +1392,7 @@
     </row>
     <row r="36" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>10</v>
@@ -1410,7 +1401,7 @@
         <v>11</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>13</v>
@@ -1421,7 +1412,7 @@
     </row>
     <row r="37" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>10</v>
@@ -1430,7 +1421,7 @@
         <v>11</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>13</v>
@@ -1441,7 +1432,7 @@
     </row>
     <row r="38" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>10</v>
@@ -1450,7 +1441,7 @@
         <v>11</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>13</v>
@@ -1461,7 +1452,7 @@
     </row>
     <row r="39" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>10</v>
@@ -1470,7 +1461,7 @@
         <v>11</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E39" s="1" t="s">
         <v>13</v>
@@ -1481,7 +1472,7 @@
     </row>
     <row r="40" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>10</v>
@@ -1490,7 +1481,7 @@
         <v>11</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E40" s="1" t="s">
         <v>13</v>
@@ -1499,9 +1490,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="41" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="41" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>10</v>
@@ -1510,7 +1501,7 @@
         <v>11</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E41" s="1" t="s">
         <v>13</v>
@@ -1521,7 +1512,7 @@
     </row>
     <row r="42" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>10</v>
@@ -1530,7 +1521,7 @@
         <v>11</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E42" s="1" t="s">
         <v>13</v>
@@ -1539,9 +1530,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="43" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="43" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>10</v>
@@ -1550,7 +1541,7 @@
         <v>11</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>13</v>
@@ -1561,7 +1552,7 @@
     </row>
     <row r="44" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>10</v>
@@ -1570,7 +1561,7 @@
         <v>11</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>13</v>
@@ -1581,7 +1572,7 @@
     </row>
     <row r="45" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>10</v>
@@ -1590,7 +1581,7 @@
         <v>11</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E45" s="1" t="s">
         <v>13</v>
@@ -1601,7 +1592,7 @@
     </row>
     <row r="46" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>10</v>
@@ -1610,7 +1601,7 @@
         <v>11</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E46" s="1" t="s">
         <v>13</v>
@@ -1621,7 +1612,7 @@
     </row>
     <row r="47" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>10</v>
@@ -1630,7 +1621,7 @@
         <v>11</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>13</v>
@@ -1641,7 +1632,7 @@
     </row>
     <row r="48" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>10</v>
@@ -1650,7 +1641,7 @@
         <v>11</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E48" s="1" t="s">
         <v>13</v>
@@ -1661,7 +1652,7 @@
     </row>
     <row r="49" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>10</v>
@@ -1670,7 +1661,7 @@
         <v>11</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E49" s="1" t="s">
         <v>13</v>
@@ -1681,7 +1672,7 @@
     </row>
     <row r="50" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>10</v>
@@ -1690,7 +1681,7 @@
         <v>11</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E50" s="1" t="s">
         <v>13</v>
@@ -1701,7 +1692,7 @@
     </row>
     <row r="51" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>10</v>
@@ -1710,7 +1701,7 @@
         <v>11</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>13</v>
@@ -1721,7 +1712,7 @@
     </row>
     <row r="52" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>10</v>
@@ -1730,7 +1721,7 @@
         <v>11</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>13</v>
@@ -1741,7 +1732,7 @@
     </row>
     <row r="53" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B53" s="1" t="s">
         <v>10</v>
@@ -1750,7 +1741,7 @@
         <v>11</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E53" s="1" t="s">
         <v>13</v>
@@ -1761,7 +1752,7 @@
     </row>
     <row r="54" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B54" s="1" t="s">
         <v>10</v>
@@ -1770,7 +1761,7 @@
         <v>11</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>13</v>
@@ -1779,48 +1770,8 @@
         <v>13</v>
       </c>
     </row>
-    <row r="55" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="B55" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="E55" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F55" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="56" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="B56" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C56" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D56" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="E56" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F56" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A5:F56"/>
+  <autoFilter ref="A5:F54"/>
   <mergeCells count="3">
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="D2:F2"/>

</xml_diff>